<commit_message>
Plan CI compatibility fix
</commit_message>
<xml_diff>
--- a/reports/BugReport.xlsx
+++ b/reports/BugReport.xlsx
@@ -463,14 +463,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
@@ -556,7 +556,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>test_login</t>
+          <t>test_delete_account</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -586,20 +586,21 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>tests/authentication/test_login.py:60: in test_login
-    assert False, "temporary failure for artifa</t>
+          <t>tests/authentication/test_delete_account.py:21: in test_delete_account
+    signup.open()
+pages/authe</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>14:33:51</t>
+          <t>08:06:06</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Expected condition not met. Verify test data and application state.</t>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -608,34 +609,949 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test_login</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>tests/authentication/test_login.py:22: in test_login
+    signup.open()
+pages/authentication/signup_p</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>08:06:07</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>test_logout</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>tests/authentication/test_logout.py:21: in test_logout
+    signup.open()
+pages/authentication/signup</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>08:06:08</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>test_register</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>tests/authentication/test_register.py:19: in test_register
+    signup.open()
+pages/authentication/si</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>08:06:09</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>test_signup</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>tests/authentication/test_signup.py:8: in test_signup
+    signup.open()
+pages/authentication/signup_</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>08:06:09</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test_continue_shopping</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_continue_shopping.py:17: in test_continue_shopping
+    product.open()
+pages/product/</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>08:06:10</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test_multiple_products</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_multiple_products.py:17: in test_multiple_products
+    product.open()
+pages/product/</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>08:06:11</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test_proceed_to_checkout</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_proceed_to_checkout.py:28: in test_proceed_to_checkout
+    signup.open()
+pages/authe</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>08:06:12</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test_remove_product</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_remove_product.py:17: in test_remove_product
+    product.open()
+pages/product/produc</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>08:06:13</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test_verify_cart_information</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_verify_cart_information.py:17: in test_verify_cart_information
+    product.open()
+pa</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>08:06:14</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test_view_cart</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Cart</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>tests/cart/test_view_cart.py:17: in test_view_cart
+    product.open()
+pages/product/product_page.py:</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>08:06:14</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test_add_to_cart</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>tests/product/test_add_to_cart.py:11: in test_add_to_cart
+    product.open()
+pages/product/product_p</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>08:06:15</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test_search_product</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>tests/product/test_search_product.py:16: in test_search_product
+    product.open()
+pages/product/pro</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>08:06:16</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test_view_products</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>tests/product/test_view_product.py:11: in test_view_products
+    product.open()
+pages/product/produc</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>08:06:17</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test_home</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>tests/smoke/test_home.py:6: in test_home
+    page.goto(BASE_URL)
+../../../.local/lib/python3.12/site</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>08:06:18</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>BUG-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test_open</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Test_open.py</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>tests/test_open.py:9: in test_open
+    browser = p.chromium.launch(
+../../../.local/lib/python3.12/s</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>08:06:18</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Network connectivity issue or server unavailable. Check network or server status.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Investigate error in detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Total Failed: 1</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Total Failed: 16</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Critical: 0</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>High: 0</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Medium: 1</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Medium: 16</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Low: 0</t>
         </is>

</xml_diff>